<commit_message>
Un poco de todo. Hago commit por seguridad
</commit_message>
<xml_diff>
--- a/data/data_preparation/auriculares/df_cust_needs.xlsx
+++ b/data/data_preparation/auriculares/df_cust_needs.xlsx
@@ -425,183 +425,133 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>cust_needs_one_word</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
           <t>cust_needs_three_words</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="n">
-        <v>0</v>
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>precio</t>
+        </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>precio</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
           <t>relacion precio calidad</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="n">
-        <v>1</v>
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>sonido</t>
+        </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>sonido</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
           <t>buena calidad sonido</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="n">
-        <v>2</v>
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>bateria</t>
+        </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>bateria</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
           <t>buena duracion bateria</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="n">
-        <v>3</v>
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>microfono</t>
+        </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>microfono</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
           <t>microfono funciona bien</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="1" t="n">
-        <v>4</v>
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>alcance</t>
+        </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>alcance</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
           <t>tiene buen alcance</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="1" t="n">
-        <v>5</v>
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>ruido</t>
+        </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>ruido</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
           <t>cancelacion ruido buena</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="1" t="n">
-        <v>6</v>
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>cable</t>
+        </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>material</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>buena calidad material</t>
+          <t>buena calidad cable</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="1" t="n">
-        <v>7</v>
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>oreja</t>
+        </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>cable</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>buena calidad cable</t>
+          <t>adaptan bien oreja</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="1" t="n">
-        <v>8</v>
+      <c r="A10" s="1" t="inlineStr">
+        <is>
+          <t>bluetooth</t>
+        </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>oreja</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>adaptan bien oreja</t>
+          <t>conexion bluetooth buena</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="1" t="n">
-        <v>9</v>
+      <c r="A11" s="1" t="inlineStr">
+        <is>
+          <t>marca</t>
+        </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>bluetooth</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>conexion bluetooth buena</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="1" t="n">
-        <v>10</v>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>diseño</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>excelente calidad diseño</t>
+          <t>ser marca reconocida</t>
         </is>
       </c>
     </row>

</xml_diff>